<commit_message>
Actualización de licitaciones 2026-10-15
</commit_message>
<xml_diff>
--- a/datos/licitaciones_en_plazo.xlsx
+++ b/datos/licitaciones_en_plazo.xlsx
@@ -768,11 +768,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A2" s="2" t="n"/>
       <c r="B2" s="3" t="n">
         <v>46310.79166666666</v>
       </c>
@@ -870,11 +866,7 @@
       <c r="Y2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A3" s="2" t="n"/>
       <c r="B3" s="3" t="n">
         <v>46310.99930555555</v>
       </c>
@@ -968,11 +960,7 @@
       <c r="Y3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="n"/>
       <c r="B4" s="3" t="n">
         <v>46311.54166666666</v>
       </c>
@@ -1062,11 +1050,7 @@
       <c r="Y4" s="2" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A5" s="2" t="n"/>
       <c r="B5" s="3" t="n">
         <v>46314.54166666666</v>
       </c>
@@ -1152,11 +1136,7 @@
       <c r="Y5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A6" s="2" t="n"/>
       <c r="B6" s="3" t="n">
         <v>46314.99930555555</v>
       </c>
@@ -1250,11 +1230,7 @@
       <c r="Y6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A7" s="2" t="n"/>
       <c r="B7" s="3" t="n">
         <v>46316.99930555555</v>
       </c>
@@ -1348,11 +1324,7 @@
       <c r="Y7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A8" s="2" t="n"/>
       <c r="B8" s="3" t="n">
         <v>46317.99930555555</v>
       </c>
@@ -1446,11 +1418,7 @@
       <c r="Y8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A9" s="2" t="n"/>
       <c r="B9" s="3" t="n">
         <v>46317.99930555555</v>
       </c>
@@ -1540,11 +1508,7 @@
       <c r="Y9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A10" s="2" t="n"/>
       <c r="B10" s="3" t="n">
         <v>46318.99930555555</v>
       </c>
@@ -1642,11 +1606,7 @@
       <c r="Y10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A11" s="2" t="n"/>
       <c r="B11" s="3" t="n">
         <v>46321.375</v>
       </c>
@@ -1740,11 +1700,7 @@
       <c r="Y11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A12" s="2" t="n"/>
       <c r="B12" s="3" t="n">
         <v>46321.54166666666</v>
       </c>
@@ -1834,11 +1790,7 @@
       <c r="Y12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A13" s="2" t="n"/>
       <c r="B13" s="3" t="n">
         <v>46321.79166666666</v>
       </c>
@@ -1928,11 +1880,7 @@
       <c r="Y13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A14" s="2" t="n"/>
       <c r="B14" s="3" t="n">
         <v>46321.99930555555</v>
       </c>
@@ -2026,11 +1974,7 @@
       <c r="Y14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A15" s="2" t="n"/>
       <c r="B15" s="3" t="n">
         <v>46321.99930555555</v>
       </c>
@@ -2124,11 +2068,7 @@
       <c r="Y15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A16" s="2" t="n"/>
       <c r="B16" s="3" t="n">
         <v>46322.99930555555</v>
       </c>
@@ -2222,11 +2162,7 @@
       <c r="Y16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A17" s="2" t="n"/>
       <c r="B17" s="3" t="n">
         <v>46322.99930555555</v>
       </c>
@@ -2320,11 +2256,7 @@
       <c r="Y17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A18" s="2" t="n"/>
       <c r="B18" s="3" t="n">
         <v>46323.04097222222</v>
       </c>
@@ -2422,11 +2354,7 @@
       <c r="Y18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A19" s="2" t="n"/>
       <c r="B19" s="3" t="n">
         <v>46323.5</v>
       </c>
@@ -2516,11 +2444,7 @@
       <c r="Y19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A20" s="2" t="n"/>
       <c r="B20" s="3" t="n">
         <v>46323.5</v>
       </c>
@@ -2610,11 +2534,7 @@
       <c r="Y20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A21" s="2" t="n"/>
       <c r="B21" s="3" t="n">
         <v>46323.5</v>
       </c>
@@ -2700,11 +2620,7 @@
       <c r="Y21" s="2" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A22" s="2" t="n"/>
       <c r="B22" s="3" t="n">
         <v>46323.99930555555</v>
       </c>
@@ -2794,11 +2710,7 @@
       <c r="Y22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A23" s="2" t="n"/>
       <c r="B23" s="3" t="n">
         <v>46323.99930555555</v>
       </c>
@@ -2896,11 +2808,7 @@
       <c r="Y23" s="2" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A24" s="2" t="n"/>
       <c r="B24" s="3" t="n">
         <v>46323.99930555555</v>
       </c>
@@ -2994,11 +2902,7 @@
       <c r="Y24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A25" s="2" t="n"/>
       <c r="B25" s="3" t="n">
         <v>46323.99930555555</v>
       </c>
@@ -3092,11 +2996,7 @@
       <c r="Y25" s="2" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A26" s="2" t="n"/>
       <c r="B26" s="3" t="n">
         <v>46324.58333333334</v>
       </c>
@@ -3186,11 +3086,7 @@
       <c r="Y26" s="2" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A27" s="2" t="n"/>
       <c r="B27" s="3" t="n">
         <v>46324.99930555555</v>
       </c>
@@ -3288,11 +3184,7 @@
       <c r="Y27" s="2" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A28" s="2" t="n"/>
       <c r="B28" s="3" t="n">
         <v>46324.99930555555</v>
       </c>
@@ -3394,11 +3286,7 @@
       <c r="Y28" s="2" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A29" s="2" t="n"/>
       <c r="B29" s="3" t="n">
         <v>46324.99930555555</v>
       </c>
@@ -3488,11 +3376,7 @@
       <c r="Y29" s="2" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A30" s="2" t="n"/>
       <c r="B30" s="3" t="n">
         <v>46325.58333333334</v>
       </c>
@@ -3582,11 +3466,7 @@
       <c r="Y30" s="2" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A31" s="2" t="n"/>
       <c r="B31" s="3" t="n">
         <v>46328.33333333334</v>
       </c>
@@ -3684,11 +3564,7 @@
       <c r="Y31" s="2" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A32" s="2" t="n"/>
       <c r="B32" s="3" t="n">
         <v>46328.58333333334</v>
       </c>
@@ -3782,11 +3658,7 @@
       <c r="Y32" s="2" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A33" s="2" t="n"/>
       <c r="B33" s="3" t="n">
         <v>46328.58333333334</v>
       </c>
@@ -3880,11 +3752,7 @@
       <c r="Y33" s="2" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A34" s="2" t="n"/>
       <c r="B34" s="3" t="n">
         <v>46328.99930555555</v>
       </c>
@@ -3978,11 +3846,7 @@
       <c r="Y34" s="2" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A35" s="2" t="n"/>
       <c r="B35" s="3" t="n">
         <v>46329.58333333334</v>
       </c>
@@ -4080,11 +3944,7 @@
       <c r="Y35" s="2" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A36" s="2" t="n"/>
       <c r="B36" s="3" t="n">
         <v>46329.79166666666</v>
       </c>
@@ -4178,11 +4038,7 @@
       <c r="Y36" s="2" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A37" s="2" t="n"/>
       <c r="B37" s="3" t="n">
         <v>46329.79166666666</v>
       </c>
@@ -4276,11 +4132,7 @@
       <c r="Y37" s="2" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A38" s="2" t="n"/>
       <c r="B38" s="3" t="n">
         <v>46329.79166666666</v>
       </c>
@@ -4374,11 +4226,7 @@
       <c r="Y38" s="2" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A39" s="2" t="n"/>
       <c r="B39" s="3" t="n">
         <v>46329.99930555555</v>
       </c>
@@ -4468,11 +4316,7 @@
       <c r="Y39" s="2" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A40" s="2" t="n"/>
       <c r="B40" s="3" t="n">
         <v>46329.99930555555</v>
       </c>
@@ -4562,11 +4406,7 @@
       <c r="Y40" s="2" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A41" s="2" t="n"/>
       <c r="B41" s="3" t="n">
         <v>46329.99930555555</v>
       </c>
@@ -4660,11 +4500,7 @@
       <c r="Y41" s="2" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A42" s="2" t="n"/>
       <c r="B42" s="3" t="n">
         <v>46329.99930555555</v>
       </c>
@@ -4754,11 +4590,7 @@
       <c r="Y42" s="2" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A43" s="2" t="n"/>
       <c r="B43" s="3" t="n">
         <v>46331.99930555555</v>
       </c>
@@ -4848,11 +4680,7 @@
       <c r="Y43" s="2" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A44" s="2" t="n"/>
       <c r="B44" s="3" t="n">
         <v>46332.99930555555</v>
       </c>
@@ -4942,11 +4770,7 @@
       <c r="Y44" s="2" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A45" s="2" t="n"/>
       <c r="B45" s="3" t="n">
         <v>46335.99930555555</v>
       </c>
@@ -5040,11 +4864,7 @@
       <c r="Y45" s="2" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A46" s="2" t="n"/>
       <c r="B46" s="3" t="n">
         <v>46335.99930555555</v>
       </c>
@@ -5146,11 +4966,7 @@
       <c r="Y46" s="2" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A47" s="2" t="n"/>
       <c r="B47" s="3" t="n">
         <v>46335.99930555555</v>
       </c>
@@ -5248,11 +5064,7 @@
       <c r="Y47" s="2" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A48" s="2" t="n"/>
       <c r="B48" s="3" t="n">
         <v>46335.99930555555</v>
       </c>
@@ -5342,11 +5154,7 @@
       <c r="Y48" s="2" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A49" s="2" t="n"/>
       <c r="B49" s="3" t="n">
         <v>46350.45833333334</v>
       </c>
@@ -5440,11 +5248,7 @@
       <c r="Y49" s="2" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
+      <c r="A50" s="2" t="n"/>
       <c r="B50" s="3" t="n">
         <v>48099.58333333334</v>
       </c>
@@ -5738,7 +5542,7 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>46310.33159722222</v>
+        <v>46310.49417824074</v>
       </c>
     </row>
     <row r="4">
@@ -5773,7 +5577,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>0 fichero(s) mensual(es) + 30 página(s) del feed</t>
+          <t>0 fichero(s) mensual(es) + 7 página(s) del feed</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5588,7 @@
         </is>
       </c>
       <c r="B7" s="14" t="n">
-        <v>14701</v>
+        <v>3226</v>
       </c>
     </row>
     <row r="8">
@@ -5795,7 +5599,7 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>06/10/2026 – 14/10/2026</t>
+          <t>13/10/2026 – 14/10/2026</t>
         </is>
       </c>
     </row>

</xml_diff>